<commit_message>
feat: add REG-009 and REG-010 Excel templates to public directory
</commit_message>
<xml_diff>
--- a/public/templates/REG-009_A_v6 ART 2.xlsx
+++ b/public/templates/REG-009_A_v6 ART 2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chico\OneDrive\Documents\Rayca\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chico\OneDrive\Documents\GitHub\FillAndSend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10FB3E18-6099-4E68-BDC4-4AB76B77E98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72AC27B-C031-46EB-87F8-A3AC0A34F6D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8EF73867-AC56-4CD5-A280-234971FB6F14}"/>
   </bookViews>
@@ -712,11 +712,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -773,6 +770,184 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -809,183 +984,13 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1368,1313 +1373,1425 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30"/>
-      <c r="B1" s="30"/>
-      <c r="C1" s="31" t="s">
+      <c r="A1" s="89"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="90" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="31"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="35" t="s">
+      <c r="D1" s="90"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="94"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30"/>
-      <c r="B2" s="30"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="35" t="s">
+      <c r="A2" s="89"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
+      <c r="G2" s="94"/>
+      <c r="H2" s="94"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="30"/>
-      <c r="B3" s="30"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="35" t="s">
+      <c r="A3" s="89"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
+      <c r="G3" s="94"/>
+      <c r="H3" s="94"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="20" t="s">
+      <c r="B4" s="92"/>
+      <c r="C4" s="92"/>
+      <c r="D4" s="92"/>
+      <c r="E4" s="92"/>
+      <c r="F4" s="93"/>
+      <c r="G4" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="20"/>
+      <c r="H4" s="19"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="26"/>
+      <c r="B5" s="87"/>
+      <c r="C5" s="88"/>
+      <c r="D5" s="83"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="85"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="28"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="3" t="s">
+      <c r="B6" s="87"/>
+      <c r="C6" s="88"/>
+      <c r="D6" s="83"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="3"/>
+      <c r="H6" s="2"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="42" t="s">
+      <c r="A7" s="81" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="42"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="43"/>
+      <c r="B7" s="81"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
+      <c r="F7" s="82"/>
+      <c r="G7" s="82"/>
+      <c r="H7" s="82"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="42"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="43"/>
+      <c r="A8" s="81"/>
+      <c r="B8" s="81"/>
+      <c r="C8" s="82"/>
+      <c r="D8" s="82"/>
+      <c r="E8" s="82"/>
+      <c r="F8" s="82"/>
+      <c r="G8" s="82"/>
+      <c r="H8" s="82"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="39"/>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="39"/>
-      <c r="H9" s="40"/>
+      <c r="B9" s="77"/>
+      <c r="C9" s="77"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="77"/>
+      <c r="F9" s="77"/>
+      <c r="G9" s="77"/>
+      <c r="H9" s="78"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="41" t="s">
+      <c r="B10" s="75"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="79" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="41"/>
+      <c r="E10" s="79"/>
+      <c r="F10" s="79"/>
+      <c r="G10" s="79"/>
+      <c r="H10" s="79"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="89" t="s">
+      <c r="A11" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="89"/>
-      <c r="C11" s="89"/>
-      <c r="D11" s="89"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="41"/>
-      <c r="G11" s="41"/>
-      <c r="H11" s="41"/>
+      <c r="B11" s="80"/>
+      <c r="C11" s="80"/>
+      <c r="D11" s="80"/>
+      <c r="E11" s="79"/>
+      <c r="F11" s="79"/>
+      <c r="G11" s="79"/>
+      <c r="H11" s="79"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="61"/>
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="4" t="s">
+      <c r="A12" s="37"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="8"/>
+      <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="92" t="s">
+      <c r="A13" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="92"/>
-      <c r="C13" s="92"/>
-      <c r="D13" s="92"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="9"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="95"/>
+      <c r="F13" s="96"/>
+      <c r="G13" s="96"/>
+      <c r="H13" s="8"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="92" t="s">
+      <c r="A14" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="92"/>
-      <c r="C14" s="92"/>
-      <c r="D14" s="92"/>
-      <c r="E14" s="90"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="9"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="95"/>
+      <c r="F14" s="96"/>
+      <c r="G14" s="96"/>
+      <c r="H14" s="8"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="92" t="s">
+      <c r="A15" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="92"/>
-      <c r="C15" s="92"/>
-      <c r="D15" s="92"/>
-      <c r="E15" s="90"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="9"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="95"/>
+      <c r="F15" s="96"/>
+      <c r="G15" s="96"/>
+      <c r="H15" s="8"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="92" t="s">
+      <c r="A16" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="92"/>
-      <c r="C16" s="92"/>
-      <c r="D16" s="92"/>
-      <c r="E16" s="90"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="9"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="95"/>
+      <c r="F16" s="96"/>
+      <c r="G16" s="96"/>
+      <c r="H16" s="8"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="92" t="s">
+      <c r="A17" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="92"/>
-      <c r="C17" s="92"/>
-      <c r="D17" s="92"/>
-      <c r="E17" s="90"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="9"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="95"/>
+      <c r="F17" s="96"/>
+      <c r="G17" s="96"/>
+      <c r="H17" s="8"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="92" t="s">
+      <c r="A18" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="92"/>
-      <c r="C18" s="92"/>
-      <c r="D18" s="92"/>
-      <c r="E18" s="90"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="9"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="95"/>
+      <c r="F18" s="96"/>
+      <c r="G18" s="96"/>
+      <c r="H18" s="8"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="92" t="s">
+      <c r="A19" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="92"/>
-      <c r="C19" s="92"/>
-      <c r="D19" s="92"/>
-      <c r="E19" s="90"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="9"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="95"/>
+      <c r="F19" s="96"/>
+      <c r="G19" s="96"/>
+      <c r="H19" s="8"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="92" t="s">
+      <c r="A20" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="92"/>
-      <c r="C20" s="92"/>
-      <c r="D20" s="92"/>
-      <c r="E20" s="91"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="9"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="97"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="8"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="92" t="s">
+      <c r="A21" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="92"/>
-      <c r="C21" s="92"/>
-      <c r="D21" s="92"/>
-      <c r="E21" s="91"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="9"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="97"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="8"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="92" t="s">
+      <c r="A22" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="92"/>
-      <c r="C22" s="92"/>
-      <c r="D22" s="92"/>
-      <c r="E22" s="91"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="9"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="97"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="8"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="92" t="s">
+      <c r="A23" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="92"/>
-      <c r="C23" s="92"/>
-      <c r="D23" s="92"/>
-      <c r="E23" s="91"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="9"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="97"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="8"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="92" t="s">
+      <c r="A24" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="92"/>
-      <c r="C24" s="92"/>
-      <c r="D24" s="92"/>
-      <c r="E24" s="91"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="9"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="97"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="8"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="92" t="s">
+      <c r="A25" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="92"/>
-      <c r="C25" s="92"/>
-      <c r="D25" s="92"/>
-      <c r="E25" s="91"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="9"/>
+      <c r="B25" s="30"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="97"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="8"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="92" t="s">
+      <c r="A26" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="92"/>
-      <c r="C26" s="92"/>
-      <c r="D26" s="92"/>
-      <c r="E26" s="91"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="9"/>
+      <c r="B26" s="30"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="97"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="8"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="92" t="s">
+      <c r="A27" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="92"/>
-      <c r="C27" s="92"/>
-      <c r="D27" s="92"/>
-      <c r="E27" s="91"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="9"/>
+      <c r="B27" s="30"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="97"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="8"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="92" t="s">
+      <c r="A28" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="92"/>
-      <c r="C28" s="92"/>
-      <c r="D28" s="92"/>
-      <c r="E28" s="91"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="9"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="8"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="92" t="s">
+      <c r="A29" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="92"/>
-      <c r="C29" s="92"/>
-      <c r="D29" s="92"/>
-      <c r="E29" s="91"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="9"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="97"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="8"/>
     </row>
     <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="44" t="s">
+      <c r="A30" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="45"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="45"/>
-      <c r="G30" s="45"/>
-      <c r="H30" s="46"/>
+      <c r="B30" s="65"/>
+      <c r="C30" s="65"/>
+      <c r="D30" s="65"/>
+      <c r="E30" s="65"/>
+      <c r="F30" s="65"/>
+      <c r="G30" s="65"/>
+      <c r="H30" s="66"/>
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="47"/>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="49"/>
+      <c r="A31" s="67"/>
+      <c r="B31" s="68"/>
+      <c r="C31" s="68"/>
+      <c r="D31" s="68"/>
+      <c r="E31" s="68"/>
+      <c r="F31" s="68"/>
+      <c r="G31" s="68"/>
+      <c r="H31" s="69"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="11"/>
-      <c r="B32" s="84" t="s">
+      <c r="A32" s="10"/>
+      <c r="B32" s="70" t="s">
         <v>35</v>
       </c>
-      <c r="C32" s="85"/>
-      <c r="D32" s="86"/>
-      <c r="E32" s="87"/>
-      <c r="F32" s="88" t="s">
+      <c r="C32" s="71"/>
+      <c r="D32" s="72"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="73" t="s">
         <v>45</v>
       </c>
-      <c r="G32" s="88"/>
-      <c r="H32" s="88"/>
+      <c r="G32" s="73"/>
+      <c r="H32" s="73"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="11"/>
-      <c r="B33" s="84" t="s">
+      <c r="A33" s="10"/>
+      <c r="B33" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="C33" s="85"/>
-      <c r="D33" s="86"/>
-      <c r="E33" s="87"/>
-      <c r="F33" s="88" t="s">
+      <c r="C33" s="71"/>
+      <c r="D33" s="72"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="73" t="s">
         <v>46</v>
       </c>
-      <c r="G33" s="88"/>
-      <c r="H33" s="88"/>
+      <c r="G33" s="73"/>
+      <c r="H33" s="73"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="11"/>
-      <c r="B34" s="84" t="s">
+      <c r="A34" s="10"/>
+      <c r="B34" s="70" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="85"/>
-      <c r="D34" s="86"/>
-      <c r="E34" s="87"/>
-      <c r="F34" s="88" t="s">
+      <c r="C34" s="71"/>
+      <c r="D34" s="72"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="G34" s="88"/>
-      <c r="H34" s="88"/>
+      <c r="G34" s="73"/>
+      <c r="H34" s="73"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="11"/>
-      <c r="B35" s="84" t="s">
+      <c r="A35" s="10"/>
+      <c r="B35" s="70" t="s">
         <v>38</v>
       </c>
-      <c r="C35" s="85"/>
-      <c r="D35" s="86"/>
-      <c r="E35" s="87"/>
-      <c r="F35" s="88" t="s">
+      <c r="C35" s="71"/>
+      <c r="D35" s="72"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="73" t="s">
         <v>48</v>
       </c>
-      <c r="G35" s="88"/>
-      <c r="H35" s="88"/>
+      <c r="G35" s="73"/>
+      <c r="H35" s="73"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="11"/>
-      <c r="B36" s="84" t="s">
+      <c r="A36" s="10"/>
+      <c r="B36" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="85"/>
-      <c r="D36" s="86"/>
-      <c r="E36" s="87"/>
-      <c r="F36" s="88" t="s">
+      <c r="C36" s="71"/>
+      <c r="D36" s="72"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="73" t="s">
         <v>49</v>
       </c>
-      <c r="G36" s="88"/>
-      <c r="H36" s="88"/>
+      <c r="G36" s="73"/>
+      <c r="H36" s="73"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="11"/>
-      <c r="B37" s="84" t="s">
+      <c r="A37" s="10"/>
+      <c r="B37" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="C37" s="85"/>
-      <c r="D37" s="86"/>
-      <c r="E37" s="87"/>
-      <c r="F37" s="88" t="s">
+      <c r="C37" s="71"/>
+      <c r="D37" s="72"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="73" t="s">
         <v>50</v>
       </c>
-      <c r="G37" s="88"/>
-      <c r="H37" s="88"/>
+      <c r="G37" s="73"/>
+      <c r="H37" s="73"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="11"/>
-      <c r="B38" s="84" t="s">
+      <c r="A38" s="10"/>
+      <c r="B38" s="70" t="s">
         <v>41</v>
       </c>
-      <c r="C38" s="85"/>
-      <c r="D38" s="86"/>
-      <c r="E38" s="87"/>
-      <c r="F38" s="88" t="s">
+      <c r="C38" s="71"/>
+      <c r="D38" s="72"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="G38" s="88"/>
-      <c r="H38" s="88"/>
+      <c r="G38" s="73"/>
+      <c r="H38" s="73"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="11"/>
-      <c r="B39" s="84" t="s">
+      <c r="A39" s="10"/>
+      <c r="B39" s="70" t="s">
         <v>42</v>
       </c>
-      <c r="C39" s="85"/>
-      <c r="D39" s="86"/>
-      <c r="E39" s="87"/>
-      <c r="F39" s="88" t="s">
+      <c r="C39" s="71"/>
+      <c r="D39" s="72"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="G39" s="88"/>
-      <c r="H39" s="88"/>
+      <c r="G39" s="73"/>
+      <c r="H39" s="73"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="11"/>
-      <c r="B40" s="84" t="s">
+      <c r="A40" s="10"/>
+      <c r="B40" s="70" t="s">
         <v>43</v>
       </c>
-      <c r="C40" s="85"/>
-      <c r="D40" s="86"/>
-      <c r="E40" s="87"/>
-      <c r="F40" s="88" t="s">
+      <c r="C40" s="71"/>
+      <c r="D40" s="72"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="73" t="s">
         <v>53</v>
       </c>
-      <c r="G40" s="88"/>
-      <c r="H40" s="88"/>
+      <c r="G40" s="73"/>
+      <c r="H40" s="73"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="11"/>
-      <c r="B41" s="84" t="s">
+      <c r="A41" s="10"/>
+      <c r="B41" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="C41" s="85"/>
-      <c r="D41" s="86"/>
-      <c r="E41" s="87"/>
-      <c r="F41" s="88" t="s">
+      <c r="C41" s="71"/>
+      <c r="D41" s="72"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="G41" s="88"/>
-      <c r="H41" s="88"/>
+      <c r="G41" s="73"/>
+      <c r="H41" s="73"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="11"/>
-      <c r="B42" s="84" t="s">
+      <c r="A42" s="10"/>
+      <c r="B42" s="70" t="s">
         <v>55</v>
       </c>
-      <c r="C42" s="85"/>
-      <c r="D42" s="86"/>
-      <c r="E42" s="87"/>
-      <c r="F42" s="88" t="s">
+      <c r="C42" s="71"/>
+      <c r="D42" s="72"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="73" t="s">
         <v>59</v>
       </c>
-      <c r="G42" s="88"/>
-      <c r="H42" s="88"/>
+      <c r="G42" s="73"/>
+      <c r="H42" s="73"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="11"/>
-      <c r="B43" s="84" t="s">
+      <c r="A43" s="10"/>
+      <c r="B43" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="C43" s="85"/>
-      <c r="D43" s="86"/>
-      <c r="E43" s="87"/>
-      <c r="F43" s="88" t="s">
+      <c r="C43" s="71"/>
+      <c r="D43" s="72"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="G43" s="88"/>
-      <c r="H43" s="88"/>
+      <c r="G43" s="73"/>
+      <c r="H43" s="73"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="11"/>
-      <c r="B44" s="84" t="s">
+      <c r="A44" s="10"/>
+      <c r="B44" s="70" t="s">
         <v>57</v>
       </c>
-      <c r="C44" s="85"/>
-      <c r="D44" s="86"/>
-      <c r="E44" s="87"/>
-      <c r="F44" s="88" t="s">
+      <c r="C44" s="71"/>
+      <c r="D44" s="72"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="73" t="s">
         <v>61</v>
       </c>
-      <c r="G44" s="88"/>
-      <c r="H44" s="88"/>
+      <c r="G44" s="73"/>
+      <c r="H44" s="73"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="11"/>
-      <c r="B45" s="84" t="s">
+      <c r="A45" s="10"/>
+      <c r="B45" s="70" t="s">
         <v>58</v>
       </c>
-      <c r="C45" s="85"/>
-      <c r="D45" s="86"/>
-      <c r="E45" s="87"/>
-      <c r="F45" s="88" t="s">
+      <c r="C45" s="71"/>
+      <c r="D45" s="72"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="73" t="s">
         <v>62</v>
       </c>
-      <c r="G45" s="88"/>
-      <c r="H45" s="88"/>
+      <c r="G45" s="73"/>
+      <c r="H45" s="73"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="11"/>
-      <c r="B46" s="84" t="s">
+      <c r="A46" s="10"/>
+      <c r="B46" s="70" t="s">
         <v>64</v>
       </c>
-      <c r="C46" s="85"/>
-      <c r="D46" s="86"/>
-      <c r="E46" s="87"/>
-      <c r="F46" s="88" t="s">
+      <c r="C46" s="71"/>
+      <c r="D46" s="72"/>
+      <c r="E46" s="24"/>
+      <c r="F46" s="73" t="s">
         <v>64</v>
       </c>
-      <c r="G46" s="88"/>
-      <c r="H46" s="88"/>
+      <c r="G46" s="73"/>
+      <c r="H46" s="73"/>
     </row>
     <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="44" t="s">
+      <c r="A47" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="B47" s="45"/>
-      <c r="C47" s="45"/>
-      <c r="D47" s="45"/>
-      <c r="E47" s="45"/>
-      <c r="F47" s="45"/>
-      <c r="G47" s="45"/>
-      <c r="H47" s="46"/>
+      <c r="B47" s="65"/>
+      <c r="C47" s="65"/>
+      <c r="D47" s="65"/>
+      <c r="E47" s="65"/>
+      <c r="F47" s="65"/>
+      <c r="G47" s="65"/>
+      <c r="H47" s="66"/>
     </row>
     <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="47"/>
-      <c r="B48" s="48"/>
-      <c r="C48" s="48"/>
-      <c r="D48" s="48"/>
-      <c r="E48" s="48"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="48"/>
-      <c r="H48" s="49"/>
+      <c r="A48" s="67"/>
+      <c r="B48" s="68"/>
+      <c r="C48" s="68"/>
+      <c r="D48" s="68"/>
+      <c r="E48" s="68"/>
+      <c r="F48" s="68"/>
+      <c r="G48" s="68"/>
+      <c r="H48" s="69"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" s="10"/>
-      <c r="B49" s="50" t="s">
+      <c r="A49" s="9"/>
+      <c r="B49" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="C49" s="50"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="50" t="s">
+      <c r="C49" s="29"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="F49" s="50"/>
-      <c r="G49" s="7"/>
-      <c r="H49" s="9"/>
+      <c r="F49" s="29"/>
+      <c r="G49" s="6"/>
+      <c r="H49" s="8"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="10"/>
-      <c r="B50" s="50" t="s">
+      <c r="A50" s="9"/>
+      <c r="B50" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="C50" s="50"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="50" t="s">
+      <c r="C50" s="29"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="F50" s="50"/>
-      <c r="G50" s="7"/>
-      <c r="H50" s="9"/>
+      <c r="F50" s="29"/>
+      <c r="G50" s="6"/>
+      <c r="H50" s="8"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="10"/>
-      <c r="B51" s="50" t="s">
+      <c r="A51" s="9"/>
+      <c r="B51" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="C51" s="50"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="50" t="s">
+      <c r="C51" s="29"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="F51" s="50"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="9"/>
+      <c r="F51" s="29"/>
+      <c r="G51" s="6"/>
+      <c r="H51" s="8"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="10"/>
-      <c r="B52" s="50" t="s">
+      <c r="A52" s="9"/>
+      <c r="B52" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="C52" s="50"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="50" t="s">
+      <c r="C52" s="29"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="F52" s="50"/>
-      <c r="G52" s="7"/>
-      <c r="H52" s="9"/>
+      <c r="F52" s="29"/>
+      <c r="G52" s="6"/>
+      <c r="H52" s="8"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A53" s="10"/>
-      <c r="B53" s="50" t="s">
+      <c r="A53" s="9"/>
+      <c r="B53" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="C53" s="50"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="50" t="s">
+      <c r="C53" s="29"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="F53" s="50"/>
-      <c r="G53" s="7"/>
-      <c r="H53" s="9"/>
+      <c r="F53" s="29"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="8"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A54" s="10"/>
-      <c r="B54" s="50" t="s">
+      <c r="A54" s="9"/>
+      <c r="B54" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="C54" s="50"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="50" t="s">
+      <c r="C54" s="29"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="F54" s="50"/>
-      <c r="G54" s="7"/>
-      <c r="H54" s="9"/>
+      <c r="F54" s="29"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="8"/>
     </row>
     <row r="55" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="53" t="s">
+      <c r="A55" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="B55" s="54"/>
-      <c r="C55" s="54"/>
-      <c r="D55" s="54"/>
-      <c r="E55" s="54"/>
-      <c r="F55" s="54"/>
-      <c r="G55" s="54"/>
-      <c r="H55" s="55"/>
+      <c r="B55" s="62"/>
+      <c r="C55" s="62"/>
+      <c r="D55" s="62"/>
+      <c r="E55" s="62"/>
+      <c r="F55" s="62"/>
+      <c r="G55" s="62"/>
+      <c r="H55" s="63"/>
     </row>
     <row r="56" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="53"/>
-      <c r="B56" s="54"/>
-      <c r="C56" s="54"/>
-      <c r="D56" s="54"/>
-      <c r="E56" s="54"/>
-      <c r="F56" s="54"/>
-      <c r="G56" s="54"/>
-      <c r="H56" s="55"/>
+      <c r="A56" s="61"/>
+      <c r="B56" s="62"/>
+      <c r="C56" s="62"/>
+      <c r="D56" s="62"/>
+      <c r="E56" s="62"/>
+      <c r="F56" s="62"/>
+      <c r="G56" s="62"/>
+      <c r="H56" s="63"/>
     </row>
     <row r="57" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="51" t="s">
+      <c r="A57" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="B57" s="51"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="52" t="s">
+      <c r="B57" s="59"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="E57" s="52"/>
-      <c r="F57" s="12"/>
-      <c r="G57" s="51" t="s">
+      <c r="E57" s="60"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="59" t="s">
         <v>86</v>
       </c>
-      <c r="H57" s="51"/>
+      <c r="H57" s="59"/>
     </row>
     <row r="58" spans="1:8" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A58" s="21" t="s">
+      <c r="A58" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="B58" s="22"/>
-      <c r="C58" s="23"/>
-      <c r="D58" s="21" t="s">
+      <c r="B58" s="21"/>
+      <c r="C58" s="22"/>
+      <c r="D58" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="E58" s="21"/>
-      <c r="F58" s="23"/>
-      <c r="G58" s="21" t="s">
+      <c r="E58" s="20"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="H58" s="21"/>
+      <c r="H58" s="20"/>
     </row>
     <row r="59" spans="1:8" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A59" s="21" t="s">
+      <c r="A59" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B59" s="22"/>
-      <c r="C59" s="23"/>
-      <c r="D59" s="21" t="s">
+      <c r="B59" s="21"/>
+      <c r="C59" s="22"/>
+      <c r="D59" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="E59" s="21"/>
-      <c r="F59" s="23"/>
-      <c r="G59" s="21" t="s">
+      <c r="E59" s="20"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="H59" s="21"/>
+      <c r="H59" s="20"/>
     </row>
     <row r="60" spans="1:8" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A60" s="21" t="s">
+      <c r="A60" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="B60" s="22"/>
-      <c r="C60" s="23"/>
-      <c r="D60" s="21" t="s">
+      <c r="B60" s="21"/>
+      <c r="C60" s="22"/>
+      <c r="D60" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="E60" s="21"/>
-      <c r="F60" s="23"/>
-      <c r="G60" s="21" t="s">
+      <c r="E60" s="20"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="H60" s="21"/>
+      <c r="H60" s="20"/>
     </row>
     <row r="61" spans="1:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="21" t="s">
+      <c r="A61" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="B61" s="22"/>
-      <c r="C61" s="23"/>
-      <c r="D61" s="21" t="s">
+      <c r="B61" s="21"/>
+      <c r="C61" s="22"/>
+      <c r="D61" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E61" s="21"/>
-      <c r="F61" s="23"/>
-      <c r="G61" s="21" t="s">
+      <c r="E61" s="20"/>
+      <c r="F61" s="22"/>
+      <c r="G61" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="H61" s="21"/>
+      <c r="H61" s="20"/>
     </row>
     <row r="62" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="21" t="s">
+      <c r="A62" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="B62" s="22"/>
-      <c r="C62" s="23"/>
-      <c r="D62" s="21" t="s">
+      <c r="B62" s="21"/>
+      <c r="C62" s="22"/>
+      <c r="D62" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E62" s="21"/>
-      <c r="F62" s="23"/>
-      <c r="G62" s="21" t="s">
+      <c r="E62" s="20"/>
+      <c r="F62" s="22"/>
+      <c r="G62" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="H62" s="21"/>
+      <c r="H62" s="20"/>
     </row>
     <row r="63" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="21" t="s">
+      <c r="A63" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="B63" s="22"/>
-      <c r="C63" s="23"/>
-      <c r="D63" s="21" t="s">
+      <c r="B63" s="21"/>
+      <c r="C63" s="22"/>
+      <c r="D63" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E63" s="21"/>
-      <c r="F63" s="23"/>
-      <c r="G63" s="21" t="s">
+      <c r="E63" s="20"/>
+      <c r="F63" s="22"/>
+      <c r="G63" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="H63" s="21"/>
+      <c r="H63" s="20"/>
     </row>
     <row r="64" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="56" t="s">
+      <c r="A64" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="B64" s="57"/>
-      <c r="C64" s="57"/>
-      <c r="D64" s="57"/>
-      <c r="E64" s="57"/>
-      <c r="F64" s="57"/>
-      <c r="G64" s="57"/>
-      <c r="H64" s="58"/>
+      <c r="B64" s="54"/>
+      <c r="C64" s="54"/>
+      <c r="D64" s="54"/>
+      <c r="E64" s="54"/>
+      <c r="F64" s="54"/>
+      <c r="G64" s="54"/>
+      <c r="H64" s="55"/>
     </row>
     <row r="65" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="56"/>
-      <c r="B65" s="57"/>
-      <c r="C65" s="57"/>
-      <c r="D65" s="57"/>
-      <c r="E65" s="57"/>
-      <c r="F65" s="57"/>
-      <c r="G65" s="57"/>
-      <c r="H65" s="58"/>
+      <c r="A65" s="53"/>
+      <c r="B65" s="54"/>
+      <c r="C65" s="54"/>
+      <c r="D65" s="54"/>
+      <c r="E65" s="54"/>
+      <c r="F65" s="54"/>
+      <c r="G65" s="54"/>
+      <c r="H65" s="55"/>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" s="93"/>
-      <c r="B66" s="94" t="s">
+      <c r="A66" s="25"/>
+      <c r="B66" s="57" t="s">
         <v>91</v>
       </c>
-      <c r="C66" s="94"/>
-      <c r="D66" s="95"/>
-      <c r="E66" s="96" t="s">
+      <c r="C66" s="57"/>
+      <c r="D66" s="26"/>
+      <c r="E66" s="58" t="s">
         <v>94</v>
       </c>
-      <c r="F66" s="96"/>
-      <c r="G66" s="96"/>
-      <c r="H66" s="13"/>
-      <c r="I66" s="2"/>
-      <c r="J66" s="2"/>
+      <c r="F66" s="58"/>
+      <c r="G66" s="58"/>
+      <c r="H66" s="12"/>
+      <c r="I66" s="1"/>
+      <c r="J66" s="1"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A67" s="93"/>
-      <c r="B67" s="94" t="s">
+      <c r="A67" s="25"/>
+      <c r="B67" s="57" t="s">
         <v>92</v>
       </c>
-      <c r="C67" s="94"/>
-      <c r="D67" s="95"/>
-      <c r="E67" s="96" t="s">
+      <c r="C67" s="57"/>
+      <c r="D67" s="26"/>
+      <c r="E67" s="58" t="s">
         <v>95</v>
       </c>
-      <c r="F67" s="96"/>
-      <c r="G67" s="96"/>
-      <c r="H67" s="13"/>
-      <c r="I67" s="2"/>
-      <c r="J67" s="2"/>
+      <c r="F67" s="58"/>
+      <c r="G67" s="58"/>
+      <c r="H67" s="12"/>
+      <c r="I67" s="1"/>
+      <c r="J67" s="1"/>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A68" s="93"/>
-      <c r="B68" s="94" t="s">
+      <c r="A68" s="25"/>
+      <c r="B68" s="57" t="s">
         <v>93</v>
       </c>
-      <c r="C68" s="94"/>
-      <c r="D68" s="95"/>
-      <c r="E68" s="96" t="s">
+      <c r="C68" s="57"/>
+      <c r="D68" s="26"/>
+      <c r="E68" s="58" t="s">
         <v>96</v>
       </c>
-      <c r="F68" s="96"/>
-      <c r="G68" s="96"/>
-      <c r="H68" s="13"/>
-      <c r="I68" s="2"/>
-      <c r="J68" s="2"/>
+      <c r="F68" s="58"/>
+      <c r="G68" s="58"/>
+      <c r="H68" s="12"/>
+      <c r="I68" s="1"/>
+      <c r="J68" s="1"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A69" s="93"/>
-      <c r="B69" s="94" t="s">
+      <c r="A69" s="25"/>
+      <c r="B69" s="57" t="s">
         <v>97</v>
       </c>
-      <c r="C69" s="94"/>
-      <c r="D69" s="93"/>
-      <c r="E69" s="96" t="s">
+      <c r="C69" s="57"/>
+      <c r="D69" s="25"/>
+      <c r="E69" s="58" t="s">
         <v>98</v>
       </c>
-      <c r="F69" s="96"/>
-      <c r="G69" s="96"/>
-      <c r="H69" s="9"/>
+      <c r="F69" s="58"/>
+      <c r="G69" s="58"/>
+      <c r="H69" s="8"/>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A70" s="93"/>
-      <c r="B70" s="94" t="s">
+      <c r="A70" s="25"/>
+      <c r="B70" s="57" t="s">
         <v>64</v>
       </c>
-      <c r="C70" s="94"/>
-      <c r="D70" s="93"/>
-      <c r="E70" s="96" t="s">
+      <c r="C70" s="57"/>
+      <c r="D70" s="25"/>
+      <c r="E70" s="58" t="s">
         <v>64</v>
       </c>
-      <c r="F70" s="96"/>
-      <c r="G70" s="96"/>
-      <c r="H70" s="9"/>
+      <c r="F70" s="58"/>
+      <c r="G70" s="58"/>
+      <c r="H70" s="8"/>
     </row>
     <row r="71" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="56" t="s">
+      <c r="A71" s="53" t="s">
         <v>99</v>
       </c>
-      <c r="B71" s="57"/>
-      <c r="C71" s="57"/>
-      <c r="D71" s="57"/>
-      <c r="E71" s="57"/>
-      <c r="F71" s="57"/>
-      <c r="G71" s="57"/>
-      <c r="H71" s="58"/>
+      <c r="B71" s="54"/>
+      <c r="C71" s="54"/>
+      <c r="D71" s="54"/>
+      <c r="E71" s="54"/>
+      <c r="F71" s="54"/>
+      <c r="G71" s="54"/>
+      <c r="H71" s="55"/>
     </row>
     <row r="72" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="56"/>
-      <c r="B72" s="57"/>
-      <c r="C72" s="57"/>
-      <c r="D72" s="57"/>
-      <c r="E72" s="57"/>
-      <c r="F72" s="57"/>
-      <c r="G72" s="57"/>
-      <c r="H72" s="58"/>
+      <c r="A72" s="53"/>
+      <c r="B72" s="54"/>
+      <c r="C72" s="54"/>
+      <c r="D72" s="54"/>
+      <c r="E72" s="54"/>
+      <c r="F72" s="54"/>
+      <c r="G72" s="54"/>
+      <c r="H72" s="55"/>
     </row>
     <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="59" t="s">
+      <c r="A73" s="56" t="s">
         <v>100</v>
       </c>
-      <c r="B73" s="59"/>
-      <c r="C73" s="59" t="s">
+      <c r="B73" s="56"/>
+      <c r="C73" s="56" t="s">
         <v>101</v>
       </c>
-      <c r="D73" s="59"/>
-      <c r="E73" s="59"/>
-      <c r="F73" s="59" t="s">
+      <c r="D73" s="56"/>
+      <c r="E73" s="56"/>
+      <c r="F73" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="G73" s="59"/>
-      <c r="H73" s="59"/>
+      <c r="G73" s="56"/>
+      <c r="H73" s="56"/>
     </row>
     <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="59"/>
-      <c r="B74" s="59"/>
-      <c r="C74" s="59"/>
-      <c r="D74" s="59"/>
-      <c r="E74" s="59"/>
-      <c r="F74" s="59"/>
-      <c r="G74" s="59"/>
-      <c r="H74" s="59"/>
+      <c r="A74" s="56"/>
+      <c r="B74" s="56"/>
+      <c r="C74" s="56"/>
+      <c r="D74" s="56"/>
+      <c r="E74" s="56"/>
+      <c r="F74" s="56"/>
+      <c r="G74" s="56"/>
+      <c r="H74" s="56"/>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A75" s="50"/>
-      <c r="B75" s="50"/>
-      <c r="C75" s="50"/>
-      <c r="D75" s="50"/>
-      <c r="E75" s="50"/>
-      <c r="F75" s="50"/>
-      <c r="G75" s="50"/>
-      <c r="H75" s="50"/>
+      <c r="A75" s="29"/>
+      <c r="B75" s="29"/>
+      <c r="C75" s="29"/>
+      <c r="D75" s="29"/>
+      <c r="E75" s="29"/>
+      <c r="F75" s="29"/>
+      <c r="G75" s="29"/>
+      <c r="H75" s="29"/>
     </row>
     <row r="76" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="56" t="s">
+      <c r="A76" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="B76" s="57"/>
-      <c r="C76" s="57"/>
-      <c r="D76" s="57"/>
-      <c r="E76" s="57"/>
-      <c r="F76" s="57"/>
-      <c r="G76" s="57"/>
-      <c r="H76" s="58"/>
+      <c r="B76" s="54"/>
+      <c r="C76" s="54"/>
+      <c r="D76" s="54"/>
+      <c r="E76" s="54"/>
+      <c r="F76" s="54"/>
+      <c r="G76" s="54"/>
+      <c r="H76" s="55"/>
     </row>
     <row r="77" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="56"/>
-      <c r="B77" s="57"/>
-      <c r="C77" s="57"/>
-      <c r="D77" s="57"/>
-      <c r="E77" s="57"/>
-      <c r="F77" s="57"/>
-      <c r="G77" s="57"/>
-      <c r="H77" s="58"/>
+      <c r="A77" s="53"/>
+      <c r="B77" s="54"/>
+      <c r="C77" s="54"/>
+      <c r="D77" s="54"/>
+      <c r="E77" s="54"/>
+      <c r="F77" s="54"/>
+      <c r="G77" s="54"/>
+      <c r="H77" s="55"/>
     </row>
     <row r="78" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="14" t="s">
+      <c r="A78" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="B78" s="73" t="s">
+      <c r="B78" s="49" t="s">
         <v>105</v>
       </c>
-      <c r="C78" s="74"/>
-      <c r="D78" s="14" t="s">
+      <c r="C78" s="50"/>
+      <c r="D78" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="E78" s="73" t="s">
+      <c r="E78" s="49" t="s">
         <v>107</v>
       </c>
-      <c r="F78" s="74"/>
-      <c r="G78" s="73" t="s">
+      <c r="F78" s="50"/>
+      <c r="G78" s="49" t="s">
         <v>108</v>
       </c>
-      <c r="H78" s="74"/>
+      <c r="H78" s="50"/>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A79" s="15"/>
-      <c r="B79" s="75"/>
-      <c r="C79" s="76"/>
-      <c r="D79" s="16"/>
-      <c r="E79" s="75"/>
-      <c r="F79" s="76"/>
-      <c r="G79" s="75"/>
-      <c r="H79" s="76"/>
+      <c r="A79" s="14"/>
+      <c r="B79" s="51"/>
+      <c r="C79" s="52"/>
+      <c r="D79" s="15"/>
+      <c r="E79" s="51"/>
+      <c r="F79" s="52"/>
+      <c r="G79" s="51"/>
+      <c r="H79" s="52"/>
     </row>
     <row r="80" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="56" t="s">
+      <c r="A80" s="53" t="s">
         <v>109</v>
       </c>
-      <c r="B80" s="57"/>
-      <c r="C80" s="57"/>
-      <c r="D80" s="57"/>
-      <c r="E80" s="57"/>
-      <c r="F80" s="57"/>
-      <c r="G80" s="57"/>
-      <c r="H80" s="58"/>
+      <c r="B80" s="54"/>
+      <c r="C80" s="54"/>
+      <c r="D80" s="54"/>
+      <c r="E80" s="54"/>
+      <c r="F80" s="54"/>
+      <c r="G80" s="54"/>
+      <c r="H80" s="55"/>
     </row>
     <row r="81" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="56"/>
-      <c r="B81" s="57"/>
-      <c r="C81" s="57"/>
-      <c r="D81" s="57"/>
-      <c r="E81" s="57"/>
-      <c r="F81" s="57"/>
-      <c r="G81" s="57"/>
-      <c r="H81" s="58"/>
+      <c r="A81" s="53"/>
+      <c r="B81" s="54"/>
+      <c r="C81" s="54"/>
+      <c r="D81" s="54"/>
+      <c r="E81" s="54"/>
+      <c r="F81" s="54"/>
+      <c r="G81" s="54"/>
+      <c r="H81" s="55"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A82" s="50" t="s">
+      <c r="A82" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="B82" s="50"/>
-      <c r="C82" s="61" t="s">
+      <c r="B82" s="29"/>
+      <c r="C82" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="D82" s="62"/>
-      <c r="E82" s="63"/>
-      <c r="F82" s="61" t="s">
+      <c r="D82" s="38"/>
+      <c r="E82" s="39"/>
+      <c r="F82" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="G82" s="62"/>
-      <c r="H82" s="63"/>
+      <c r="G82" s="38"/>
+      <c r="H82" s="39"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A83" s="60"/>
-      <c r="B83" s="60"/>
-      <c r="C83" s="64"/>
-      <c r="D83" s="65"/>
-      <c r="E83" s="66"/>
-      <c r="F83" s="64"/>
-      <c r="G83" s="65"/>
-      <c r="H83" s="66"/>
+      <c r="A83" s="36"/>
+      <c r="B83" s="36"/>
+      <c r="C83" s="40"/>
+      <c r="D83" s="41"/>
+      <c r="E83" s="42"/>
+      <c r="F83" s="40"/>
+      <c r="G83" s="41"/>
+      <c r="H83" s="42"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A84" s="60"/>
-      <c r="B84" s="60"/>
-      <c r="C84" s="67"/>
-      <c r="D84" s="68"/>
-      <c r="E84" s="69"/>
-      <c r="F84" s="67"/>
-      <c r="G84" s="68"/>
-      <c r="H84" s="69"/>
+      <c r="A84" s="36"/>
+      <c r="B84" s="36"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="44"/>
+      <c r="E84" s="45"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="44"/>
+      <c r="H84" s="45"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A85" s="60"/>
-      <c r="B85" s="60"/>
-      <c r="C85" s="70"/>
-      <c r="D85" s="71"/>
-      <c r="E85" s="72"/>
-      <c r="F85" s="70"/>
-      <c r="G85" s="71"/>
-      <c r="H85" s="72"/>
+      <c r="A85" s="36"/>
+      <c r="B85" s="36"/>
+      <c r="C85" s="46"/>
+      <c r="D85" s="47"/>
+      <c r="E85" s="48"/>
+      <c r="F85" s="46"/>
+      <c r="G85" s="47"/>
+      <c r="H85" s="48"/>
     </row>
     <row r="86" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="77" t="s">
+      <c r="A86" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="B86" s="77"/>
-      <c r="C86" s="77"/>
-      <c r="D86" s="77"/>
-      <c r="E86" s="77"/>
-      <c r="F86" s="77"/>
-      <c r="G86" s="77"/>
-      <c r="H86" s="77"/>
+      <c r="B86" s="27"/>
+      <c r="C86" s="27"/>
+      <c r="D86" s="27"/>
+      <c r="E86" s="27"/>
+      <c r="F86" s="27"/>
+      <c r="G86" s="27"/>
+      <c r="H86" s="27"/>
     </row>
     <row r="87" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="77"/>
-      <c r="B87" s="77"/>
-      <c r="C87" s="77"/>
-      <c r="D87" s="77"/>
-      <c r="E87" s="77"/>
-      <c r="F87" s="77"/>
-      <c r="G87" s="77"/>
-      <c r="H87" s="77"/>
+      <c r="A87" s="27"/>
+      <c r="B87" s="27"/>
+      <c r="C87" s="27"/>
+      <c r="D87" s="27"/>
+      <c r="E87" s="27"/>
+      <c r="F87" s="27"/>
+      <c r="G87" s="27"/>
+      <c r="H87" s="27"/>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A88" s="17"/>
-      <c r="B88" s="78" t="s">
+      <c r="A88" s="16"/>
+      <c r="B88" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="C88" s="78"/>
-      <c r="D88" s="17"/>
-      <c r="E88" s="78" t="s">
+      <c r="C88" s="31"/>
+      <c r="D88" s="16"/>
+      <c r="E88" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="F88" s="78"/>
-      <c r="G88" s="7"/>
-      <c r="H88" s="9"/>
+      <c r="F88" s="31"/>
+      <c r="G88" s="6"/>
+      <c r="H88" s="8"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A89" s="18"/>
-      <c r="B89" s="79" t="s">
+      <c r="A89" s="17"/>
+      <c r="B89" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="C89" s="79"/>
-      <c r="D89" s="18"/>
-      <c r="E89" s="81" t="s">
+      <c r="C89" s="32"/>
+      <c r="D89" s="17"/>
+      <c r="E89" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="F89" s="81"/>
-      <c r="G89" s="7"/>
-      <c r="H89" s="9"/>
+      <c r="F89" s="34"/>
+      <c r="G89" s="6"/>
+      <c r="H89" s="8"/>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A90" s="18"/>
-      <c r="B90" s="79" t="s">
+      <c r="A90" s="17"/>
+      <c r="B90" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="C90" s="79"/>
-      <c r="D90" s="18"/>
-      <c r="E90" s="81" t="s">
+      <c r="C90" s="32"/>
+      <c r="D90" s="17"/>
+      <c r="E90" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="F90" s="81"/>
-      <c r="G90" s="7"/>
-      <c r="H90" s="9"/>
+      <c r="F90" s="34"/>
+      <c r="G90" s="6"/>
+      <c r="H90" s="8"/>
     </row>
     <row r="91" spans="1:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="18"/>
-      <c r="B91" s="79" t="s">
+      <c r="A91" s="17"/>
+      <c r="B91" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="C91" s="79"/>
-      <c r="D91" s="18"/>
-      <c r="E91" s="79" t="s">
+      <c r="C91" s="32"/>
+      <c r="D91" s="17"/>
+      <c r="E91" s="32" t="s">
         <v>121</v>
       </c>
-      <c r="F91" s="79"/>
-      <c r="G91" s="7"/>
-      <c r="H91" s="9"/>
+      <c r="F91" s="32"/>
+      <c r="G91" s="6"/>
+      <c r="H91" s="8"/>
     </row>
     <row r="92" spans="1:8" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="19"/>
-      <c r="B92" s="80" t="s">
+      <c r="A92" s="18"/>
+      <c r="B92" s="33" t="s">
         <v>122</v>
       </c>
-      <c r="C92" s="80"/>
-      <c r="D92" s="19"/>
-      <c r="E92" s="82" t="s">
+      <c r="C92" s="33"/>
+      <c r="D92" s="18"/>
+      <c r="E92" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="F92" s="82"/>
-      <c r="G92" s="7"/>
-      <c r="H92" s="9"/>
+      <c r="F92" s="35"/>
+      <c r="G92" s="6"/>
+      <c r="H92" s="8"/>
     </row>
     <row r="93" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="77" t="s">
+      <c r="A93" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="B93" s="77"/>
-      <c r="C93" s="77"/>
-      <c r="D93" s="77"/>
-      <c r="E93" s="77"/>
-      <c r="F93" s="77"/>
-      <c r="G93" s="77"/>
-      <c r="H93" s="77"/>
+      <c r="B93" s="27"/>
+      <c r="C93" s="27"/>
+      <c r="D93" s="27"/>
+      <c r="E93" s="27"/>
+      <c r="F93" s="27"/>
+      <c r="G93" s="27"/>
+      <c r="H93" s="27"/>
     </row>
     <row r="94" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="77"/>
-      <c r="B94" s="77"/>
-      <c r="C94" s="77"/>
-      <c r="D94" s="77"/>
-      <c r="E94" s="77"/>
-      <c r="F94" s="77"/>
-      <c r="G94" s="77"/>
-      <c r="H94" s="77"/>
+      <c r="A94" s="27"/>
+      <c r="B94" s="27"/>
+      <c r="C94" s="27"/>
+      <c r="D94" s="27"/>
+      <c r="E94" s="27"/>
+      <c r="F94" s="27"/>
+      <c r="G94" s="27"/>
+      <c r="H94" s="27"/>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A95" s="83"/>
-      <c r="B95" s="83"/>
-      <c r="C95" s="83"/>
-      <c r="D95" s="83"/>
-      <c r="E95" s="83"/>
-      <c r="F95" s="83"/>
-      <c r="G95" s="83"/>
-      <c r="H95" s="83"/>
+      <c r="A95" s="28"/>
+      <c r="B95" s="28"/>
+      <c r="C95" s="28"/>
+      <c r="D95" s="28"/>
+      <c r="E95" s="28"/>
+      <c r="F95" s="28"/>
+      <c r="G95" s="28"/>
+      <c r="H95" s="28"/>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A96" s="83"/>
-      <c r="B96" s="83"/>
-      <c r="C96" s="83"/>
-      <c r="D96" s="83"/>
-      <c r="E96" s="83"/>
-      <c r="F96" s="83"/>
-      <c r="G96" s="83"/>
-      <c r="H96" s="83"/>
+      <c r="A96" s="28"/>
+      <c r="B96" s="28"/>
+      <c r="C96" s="28"/>
+      <c r="D96" s="28"/>
+      <c r="E96" s="28"/>
+      <c r="F96" s="28"/>
+      <c r="G96" s="28"/>
+      <c r="H96" s="28"/>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A97" s="83"/>
-      <c r="B97" s="83"/>
-      <c r="C97" s="83"/>
-      <c r="D97" s="83"/>
-      <c r="E97" s="83"/>
-      <c r="F97" s="83"/>
-      <c r="G97" s="83"/>
-      <c r="H97" s="83"/>
+      <c r="A97" s="28"/>
+      <c r="B97" s="28"/>
+      <c r="C97" s="28"/>
+      <c r="D97" s="28"/>
+      <c r="E97" s="28"/>
+      <c r="F97" s="28"/>
+      <c r="G97" s="28"/>
+      <c r="H97" s="28"/>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A98" s="83"/>
-      <c r="B98" s="83"/>
-      <c r="C98" s="83"/>
-      <c r="D98" s="83"/>
-      <c r="E98" s="83"/>
-      <c r="F98" s="83"/>
-      <c r="G98" s="83"/>
-      <c r="H98" s="83"/>
+      <c r="A98" s="28"/>
+      <c r="B98" s="28"/>
+      <c r="C98" s="28"/>
+      <c r="D98" s="28"/>
+      <c r="E98" s="28"/>
+      <c r="F98" s="28"/>
+      <c r="G98" s="28"/>
+      <c r="H98" s="28"/>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A99" s="50"/>
-      <c r="B99" s="50"/>
-      <c r="C99" s="50"/>
-      <c r="D99" s="50"/>
-      <c r="E99" s="50"/>
-      <c r="F99" s="50"/>
-      <c r="G99" s="50"/>
-      <c r="H99" s="50"/>
+      <c r="A99" s="29"/>
+      <c r="B99" s="29"/>
+      <c r="C99" s="29"/>
+      <c r="D99" s="29"/>
+      <c r="E99" s="29"/>
+      <c r="F99" s="29"/>
+      <c r="G99" s="29"/>
+      <c r="H99" s="29"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A100" s="50"/>
-      <c r="B100" s="50"/>
-      <c r="C100" s="50"/>
-      <c r="D100" s="50"/>
-      <c r="E100" s="50"/>
-      <c r="F100" s="50"/>
-      <c r="G100" s="50"/>
-      <c r="H100" s="50"/>
+      <c r="A100" s="29"/>
+      <c r="B100" s="29"/>
+      <c r="C100" s="29"/>
+      <c r="D100" s="29"/>
+      <c r="E100" s="29"/>
+      <c r="F100" s="29"/>
+      <c r="G100" s="29"/>
+      <c r="H100" s="29"/>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A101" s="50"/>
-      <c r="B101" s="50"/>
-      <c r="C101" s="50"/>
-      <c r="D101" s="50"/>
-      <c r="E101" s="50"/>
-      <c r="F101" s="50"/>
-      <c r="G101" s="50"/>
-      <c r="H101" s="50"/>
+      <c r="A101" s="29"/>
+      <c r="B101" s="29"/>
+      <c r="C101" s="29"/>
+      <c r="D101" s="29"/>
+      <c r="E101" s="29"/>
+      <c r="F101" s="29"/>
+      <c r="G101" s="29"/>
+      <c r="H101" s="29"/>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A102" s="50" t="s">
+      <c r="A102" s="29" t="s">
         <v>124</v>
       </c>
-      <c r="B102" s="50"/>
-      <c r="C102" s="50"/>
-      <c r="D102" s="50" t="s">
+      <c r="B102" s="29"/>
+      <c r="C102" s="29"/>
+      <c r="D102" s="29" t="s">
         <v>107</v>
       </c>
-      <c r="E102" s="50"/>
-      <c r="F102" s="50" t="s">
+      <c r="E102" s="29"/>
+      <c r="F102" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="G102" s="50"/>
-      <c r="H102" s="50"/>
+      <c r="G102" s="29"/>
+      <c r="H102" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="136">
+    <mergeCell ref="A7:B8"/>
+    <mergeCell ref="C7:H8"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:E3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A30:H31"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="F37:H37"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="F38:H38"/>
+    <mergeCell ref="F39:H39"/>
+    <mergeCell ref="A47:H48"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="F46:H46"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="F41:H41"/>
+    <mergeCell ref="F42:H42"/>
+    <mergeCell ref="F43:H43"/>
+    <mergeCell ref="F44:H44"/>
+    <mergeCell ref="F45:H45"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="E54:F54"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="A55:H56"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="E53:F53"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="A64:H65"/>
+    <mergeCell ref="C73:E74"/>
+    <mergeCell ref="F73:H74"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="F75:H75"/>
+    <mergeCell ref="E66:G66"/>
+    <mergeCell ref="E67:G67"/>
+    <mergeCell ref="A76:H77"/>
+    <mergeCell ref="A73:B74"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="A71:H72"/>
+    <mergeCell ref="A80:H81"/>
+    <mergeCell ref="E68:G68"/>
+    <mergeCell ref="E69:G69"/>
+    <mergeCell ref="E70:G70"/>
+    <mergeCell ref="A82:B82"/>
+    <mergeCell ref="A83:B85"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="F82:H82"/>
+    <mergeCell ref="C83:E85"/>
+    <mergeCell ref="F83:H85"/>
+    <mergeCell ref="G78:H78"/>
+    <mergeCell ref="E78:F78"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="E79:F79"/>
+    <mergeCell ref="G79:H79"/>
+    <mergeCell ref="A86:H87"/>
+    <mergeCell ref="B88:C88"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="E88:F88"/>
+    <mergeCell ref="E89:F89"/>
+    <mergeCell ref="E90:F90"/>
+    <mergeCell ref="E91:F91"/>
+    <mergeCell ref="E92:F92"/>
     <mergeCell ref="A93:H94"/>
     <mergeCell ref="A95:H98"/>
     <mergeCell ref="A99:C101"/>
@@ -2699,118 +2816,6 @@
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A86:H87"/>
-    <mergeCell ref="B88:C88"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B90:C90"/>
-    <mergeCell ref="B91:C91"/>
-    <mergeCell ref="B92:C92"/>
-    <mergeCell ref="E88:F88"/>
-    <mergeCell ref="E89:F89"/>
-    <mergeCell ref="E90:F90"/>
-    <mergeCell ref="E91:F91"/>
-    <mergeCell ref="E92:F92"/>
-    <mergeCell ref="A82:B82"/>
-    <mergeCell ref="A83:B85"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="F82:H82"/>
-    <mergeCell ref="C83:E85"/>
-    <mergeCell ref="F83:H85"/>
-    <mergeCell ref="G78:H78"/>
-    <mergeCell ref="E78:F78"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="E79:F79"/>
-    <mergeCell ref="G79:H79"/>
-    <mergeCell ref="A76:H77"/>
-    <mergeCell ref="A73:B74"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="A71:H72"/>
-    <mergeCell ref="A80:H81"/>
-    <mergeCell ref="E68:G68"/>
-    <mergeCell ref="E69:G69"/>
-    <mergeCell ref="E70:G70"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="A64:H65"/>
-    <mergeCell ref="C73:E74"/>
-    <mergeCell ref="F73:H74"/>
-    <mergeCell ref="A75:B75"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="F75:H75"/>
-    <mergeCell ref="E66:G66"/>
-    <mergeCell ref="E67:G67"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="G57:H57"/>
-    <mergeCell ref="E54:F54"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="A55:H56"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="E52:F52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="E53:F53"/>
-    <mergeCell ref="A47:H48"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="F46:H46"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="E50:F50"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="F41:H41"/>
-    <mergeCell ref="F42:H42"/>
-    <mergeCell ref="F43:H43"/>
-    <mergeCell ref="F44:H44"/>
-    <mergeCell ref="F45:H45"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="F33:H33"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="F37:H37"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="F38:H38"/>
-    <mergeCell ref="F39:H39"/>
-    <mergeCell ref="A30:H31"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:H10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:H11"/>
-    <mergeCell ref="A7:B8"/>
-    <mergeCell ref="C7:H8"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:E3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="D6:F6"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>